<commit_message>
docs(STT-20): chốt đặc tả tấn công T1–T8 và phòng thủ D1–D4, đồng bộ kế hoạch
Đặc tả STT-20 (phần tài liệu):
- payload_taxonomy.md: T1–T8, cây quyết định gán nhãn, schema payload, activation_check
  theo G1/G2/G3. Chốt schema: goal_binding bắt buộc có điều kiện; base_frame giữ (T8 bắt
  buộc, T6/T7 khuyến nghị), T4 ngoài tập (không chồng cơ chế né); T2×K2a giữ cho.
- defense_spec.md: D1–D4 (chữ ký hàm, thuật toán, luật R1–R4/E1–E4, hit vào trace).
- payload_author_worksheet.md + HUONG_DAN_DIEN_PAYLOAD.md: khung điền và hướng dẫn soạn.

Nới bất biến 6 (xử VT-3): goal_binding.tool = None khi G3 hoặc khi G1 rò chỉ qua
final_answer (bồn G1 duy nhất của CT-01/02/03, không có tool-call).

Đồng bộ: Kế hoạch STT-20 → "Xong (đặc tả)"; Lộ trình thêm schema payload + validator vào
"Đã có". Phần tập payload đầy đủ + pilot + khóa v-attack-1.0 chờ lõi agent STT-26.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Kế hoạch thực hiện.xlsx
+++ b/Kế hoạch thực hiện.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="680" windowWidth="29400" windowHeight="18440" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Kế hoạch chi tiết" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Tổng quan mốc" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Khối lượng giờ" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Báo cáo 2 tuần" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kế hoạch chi tiết" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan mốc" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Khối lượng giờ" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Báo cáo 2 tuần" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Kế hoạch chi tiết'!$A$1:$K$104</definedName>
@@ -1503,49 +1503,15 @@
       </c>
     </row>
     <row r="17" ht="30" customHeight="1" s="36">
-      <c r="A17" s="21" t="n">
-        <v>14</v>
-      </c>
-      <c r="B17" s="21" t="inlineStr">
-        <is>
-          <t>ND2</t>
-        </is>
-      </c>
-      <c r="C17" s="21" t="inlineStr">
-        <is>
-          <t>Tuần 5</t>
-        </is>
-      </c>
-      <c r="D17" s="24" t="inlineStr">
-        <is>
-          <t>Chốt tên chính xác 3 model đích: A1 frontier / A2 lớp doanh nghiệp Việt / A3 lớp rẻ. Thêm khối targets vào config/models.yaml + .env, KHÔNG sửa code</t>
-        </is>
-      </c>
-      <c r="E17" s="24" t="inlineStr">
-        <is>
-          <t>config/models.yaml + .env</t>
-        </is>
-      </c>
-      <c r="F17" s="21" t="inlineStr">
-        <is>
-          <t>05/10/2026</t>
-        </is>
-      </c>
-      <c r="G17" s="21" t="inlineStr">
-        <is>
-          <t>11/10/2026</t>
-        </is>
-      </c>
-      <c r="H17" s="21" t="inlineStr">
-        <is>
-          <t>Xong</t>
-        </is>
-      </c>
-      <c r="I17" s="24" t="inlineStr">
-        <is>
-          <t>Xong thì git tag v-models-1.0. Không đổi model sau mốc này</t>
-        </is>
-      </c>
+      <c r="A17" s="20" t="n"/>
+      <c r="B17" s="20" t="n"/>
+      <c r="C17" s="20" t="n"/>
+      <c r="D17" s="23" t="n"/>
+      <c r="E17" s="23" t="n"/>
+      <c r="F17" s="20" t="n"/>
+      <c r="G17" s="20" t="n"/>
+      <c r="H17" s="20" t="n"/>
+      <c r="I17" s="23" t="n"/>
       <c r="J17" s="26" t="inlineStr">
         <is>
           <t>Claude soạn khối targets trong models.yaml và .env.example; không đụng .env thật.</t>
@@ -1556,49 +1522,15 @@
       </c>
     </row>
     <row r="18" ht="30" customHeight="1" s="36">
-      <c r="A18" s="21" t="n">
-        <v>15</v>
-      </c>
-      <c r="B18" s="21" t="inlineStr">
-        <is>
-          <t>ND2</t>
-        </is>
-      </c>
-      <c r="C18" s="21" t="inlineStr">
-        <is>
-          <t>Tuần 5</t>
-        </is>
-      </c>
-      <c r="D18" s="24" t="inlineStr">
-        <is>
-          <t>Tra giá thật A1/A2/A3 trên dashboard gateway, điền cost_budget.md §3 và §5, đặt hard cap và cảnh báo ở mức 80% hạn mức</t>
-        </is>
-      </c>
-      <c r="E18" s="24" t="inlineStr">
-        <is>
-          <t>docs/cost_budget.md (§3, §5)</t>
-        </is>
-      </c>
-      <c r="F18" s="21" t="inlineStr">
-        <is>
-          <t>05/10/2026</t>
-        </is>
-      </c>
-      <c r="G18" s="21" t="inlineStr">
-        <is>
-          <t>11/10/2026</t>
-        </is>
-      </c>
-      <c r="H18" s="21" t="inlineStr">
-        <is>
-          <t>Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="I18" s="24" t="inlineStr">
-        <is>
-          <t>Bắt buộc trước khi chạy bất kỳ lô nào. Không mở/sửa .env thay người dùng</t>
-        </is>
-      </c>
+      <c r="A18" s="20" t="n"/>
+      <c r="B18" s="20" t="n"/>
+      <c r="C18" s="20" t="n"/>
+      <c r="D18" s="23" t="n"/>
+      <c r="E18" s="23" t="n"/>
+      <c r="F18" s="20" t="n"/>
+      <c r="G18" s="20" t="n"/>
+      <c r="H18" s="20" t="n"/>
+      <c r="I18" s="23" t="n"/>
       <c r="J18" s="26" t="inlineStr">
         <is>
           <t>Claude dựng bảng tính chi phí theo công thức; TA tra đơn giá thật trên dashboard.</t>
@@ -1678,45 +1610,45 @@
       <c r="J20" s="34" t="n"/>
     </row>
     <row r="21" ht="30" customHeight="1" s="36">
-      <c r="A21" s="21" t="n">
+      <c r="A21" s="20" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="21" t="inlineStr">
+      <c r="B21" s="20" t="inlineStr">
         <is>
           <t>ND3</t>
         </is>
       </c>
-      <c r="C21" s="21" t="inlineStr">
+      <c r="C21" s="20" t="inlineStr">
         <is>
           <t>Tuần 6</t>
         </is>
       </c>
-      <c r="D21" s="24" t="inlineStr">
+      <c r="D21" s="23" t="inlineStr">
         <is>
           <t>Thiết kế kiến trúc testbed 5 tầng: lõi agent · tầng công cụ MCP · kho tri thức · tầng phòng thủ · tầng đo lường; định nghĩa điểm móc (hook) để cắm phòng thủ</t>
         </is>
       </c>
-      <c r="E21" s="24" t="inlineStr">
+      <c r="E21" s="23" t="inlineStr">
         <is>
           <t>Hình kiến trúc + đặc tả interface</t>
         </is>
       </c>
-      <c r="F21" s="21" t="inlineStr">
+      <c r="F21" s="20" t="inlineStr">
         <is>
           <t>12/10/2026</t>
         </is>
       </c>
-      <c r="G21" s="21" t="inlineStr">
+      <c r="G21" s="20" t="inlineStr">
         <is>
           <t>18/10/2026</t>
         </is>
       </c>
-      <c r="H21" s="21" t="inlineStr">
-        <is>
-          <t>Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="I21" s="24" t="inlineStr">
+      <c r="H21" s="20" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="I21" s="23" t="inlineStr">
         <is>
           <t>config/ là hợp đồng, viết trước src/</t>
         </is>
@@ -1771,7 +1703,7 @@
       </c>
       <c r="I22" s="23" t="inlineStr">
         <is>
-          <t>ĐÃ KHOÁ bằng tag v-bench-1.0 — QUY TẮC CỨNG #1: không sửa</t>
+          <t>QUY TẮC CỨNG #1: không sửa/khóa theo quy tắc cứng #1</t>
         </is>
       </c>
       <c r="J22" s="26" t="inlineStr">
@@ -1870,12 +1802,16 @@
           <t>25/10/2026</t>
         </is>
       </c>
-      <c r="H24" s="21" t="inlineStr">
-        <is>
-          <t>Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="I24" s="24" t="n"/>
+      <c r="H24" s="20" t="inlineStr">
+        <is>
+          <t>Xong (đặc tả)</t>
+        </is>
+      </c>
+      <c r="I24" s="24" t="inlineStr">
+        <is>
+          <t>Đặc tả T1–T8 + D1–D4 xong (payload_taxonomy.md, defense_spec.md). Phần code: validator schema.py + 17 payload mẫu (đủ 8 kỹ thuật) + worksheet + hướng dẫn, validate 20 test xanh. CÒN: GVHD rà câu chữ payload; tập payload đầy đủ + pilot defense=OFF (chặn bởi lõi agent STT-26) + gán nhãn kép κ≥0,80 + khóa v-attack-1.0.</t>
+        </is>
+      </c>
       <c r="J24" s="26" t="inlineStr">
         <is>
           <t>Claude viết đặc tả T1–T8, D1–D4 theo một mẫu thống nhất; TA chốt ranh giới để không trùng.</t>

</xml_diff>